<commit_message>
added CB to example
</commit_message>
<xml_diff>
--- a/annotators/teddy-4929.example.xlsx
+++ b/annotators/teddy-4929.example.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1930" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1960" uniqueCount="810">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -992,7 +992,7 @@
     <t xml:space="preserve">def-np.dem</t>
   </si>
   <si>
-    <t xml:space="preserve">syntactic focus of last sentence (post-positioned)</t>
+    <t xml:space="preserve">FOCUS: syntactic focus of last sentence (post-positioned); CB: object of main clause, hence &gt; destroyer (subject of subordinate clause)</t>
   </si>
   <si>
     <t xml:space="preserve">hunted</t>
@@ -1058,7 +1058,7 @@
     <t xml:space="preserve">Unsinkable</t>
   </si>
   <si>
-    <t xml:space="preserve">parser took “Unsinkable” as syntactic head of “Unsinkable Sam”; IN_FOCUS because mentioned in both preceding sentences</t>
+    <t xml:space="preserve">parser took “Unsinkable” as syntactic head of “Unsinkable Sam”; IN_FOCUS because mentioned in both preceding sentences; CB: we skip the preceding fragment</t>
   </si>
   <si>
     <t xml:space="preserve">Sam</t>
@@ -1349,7 +1349,7 @@
     <t xml:space="preserve">house</t>
   </si>
   <si>
-    <t xml:space="preserve">so far, we described these as cats, but we only talked about house cats</t>
+    <t xml:space="preserve">so far, we described these as cats, but we only talked about house cats; CB: guidelines formulated for entity references, hence, we do not annotate “domestication”</t>
   </si>
   <si>
     <t xml:space="preserve">can</t>
@@ -1472,6 +1472,9 @@
     <t xml:space="preserve">These</t>
   </si>
   <si>
+    <t xml:space="preserve">CB: only recurring referent</t>
+  </si>
+  <si>
     <t xml:space="preserve">stored</t>
   </si>
   <si>
@@ -1520,7 +1523,7 @@
     <t xml:space="preserve">GROUP</t>
   </si>
   <si>
-    <t xml:space="preserve">all group members are previously mentioned</t>
+    <t xml:space="preserve">all group members are previously mentioned; CB: as we annotate a group reference, this is a recurring entity</t>
   </si>
   <si>
     <t xml:space="preserve">attracted</t>
@@ -2255,7 +2258,7 @@
     <t xml:space="preserve">fs_lybica_lineages&gt;eg_cat,fs_lybica</t>
   </si>
   <si>
-    <t xml:space="preserve">eg_cats is IN FOCUS, but Anatolian cats (the first instance case of “fs_lybica”) is FAMILIAR, only</t>
+    <t xml:space="preserve">eg_cats is IN FOCUS, but Anatolian cats (the first instance case of “fs_lybica”) is FAMILIAR, only; no CB because “fs_lybica” doesn’t appear in the preceding sentence</t>
   </si>
   <si>
     <t xml:space="preserve">probably</t>
@@ -2265,6 +2268,9 @@
   </si>
   <si>
     <t xml:space="preserve">point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">only recurring referent, hence CB</t>
   </si>
   <si>
     <t xml:space="preserve">continued</t>
@@ -2648,7 +2654,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2768,10 +2774,6 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4261,8 +4263,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.96"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="9" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="40.71"/>
   </cols>
@@ -5676,9 +5678,8 @@
       <c r="G42" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H42" s="25" t="str">
-        <f aca="false">IF(J42&lt;&gt;1,"",IF(I42="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H42" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I42" s="26" t="str">
         <f aca="false">IF(OR(E42="",E42="!!!",F42="NEW"),"",INDEX(B13:B$30,-1+SUMPRODUCT(MAX(ROW(E13:E$30)*(E42=E13:E$30)))))</f>
@@ -6479,7 +6480,7 @@
       </c>
       <c r="L66" s="27"/>
     </row>
-    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="21" t="s">
         <v>38</v>
       </c>
@@ -6502,9 +6503,8 @@
       <c r="G67" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H67" s="25" t="str">
-        <f aca="false">IF(J67&lt;&gt;1,"",IF(I67="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H67" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I67" s="26" t="str">
         <f aca="false">IF(OR(E67="",E67="!!!",F67="NEW"),"",INDEX(B8:B$60,-1+SUMPRODUCT(MAX(ROW(E8:E$60)*(E67=E8:E$60)))))</f>
@@ -7473,9 +7473,8 @@
       <c r="G96" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H96" s="25" t="str">
-        <f aca="false">IF(J96&lt;&gt;1,"",IF(I96="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H96" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I96" s="26" t="str">
         <f aca="false">IF(OR(E96="",E96="!!!",F96="NEW"),"",INDEX(B8:B$89,-1+SUMPRODUCT(MAX(ROW(E8:E$89)*(E96=E8:E$89)))))</f>
@@ -7585,7 +7584,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="21" t="s">
         <v>333</v>
       </c>
@@ -7608,9 +7607,8 @@
       <c r="G103" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H103" s="25" t="str">
-        <f aca="false">IF(J103&lt;&gt;1,"",IF(I103="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H103" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I103" s="26" t="str">
         <f aca="false">IF(OR(E103="",E103="!!!",F103="NEW"),"",INDEX(B2:B$102,-1+SUMPRODUCT(MAX(ROW(E2:E$102)*(E103=E2:E$102)))))</f>
@@ -9576,9 +9574,8 @@
       <c r="G162" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H162" s="25" t="str">
-        <f aca="false">IF(J162&lt;&gt;1,"",IF(I162="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H162" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I162" s="26" t="str">
         <f aca="false">IF(OR(E162="",E162="!!!",F162="NEW"),"",INDEX(B3:B$160,-1+SUMPRODUCT(MAX(ROW(E3:E$160)*(E162=E3:E$160)))))</f>
@@ -10518,9 +10515,8 @@
       <c r="G190" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H190" s="25" t="str">
-        <f aca="false">IF(J190&lt;&gt;1,"",IF(I190="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H190" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I190" s="26" t="str">
         <f aca="false">IF(OR(E190="",E190="!!!",F190="NEW"),"",INDEX(B7:B$184,-1+SUMPRODUCT(MAX(ROW(E7:E$184)*(E190=E7:E$184)))))</f>
@@ -11144,7 +11140,7 @@
       </c>
       <c r="L209" s="27"/>
     </row>
-    <row r="210" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="21" t="s">
         <v>38</v>
       </c>
@@ -11167,9 +11163,8 @@
       <c r="G210" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H210" s="25" t="str">
-        <f aca="false">IF(J210&lt;&gt;1,"",IF(I210="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H210" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I210" s="26" t="str">
         <f aca="false">IF(OR(E210="",E210="!!!",F210="NEW"),"",INDEX(B8:B$203,-1+SUMPRODUCT(MAX(ROW(E8:E$203)*(E210=E8:E$203)))))</f>
@@ -12895,9 +12890,8 @@
       <c r="G262" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H262" s="25" t="str">
-        <f aca="false">IF(J262&lt;&gt;1,"",IF(I262="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H262" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I262" s="26" t="str">
         <f aca="false">IF(OR(E262="",E262="!!!",F262="NEW"),"",INDEX(B4:B$259,-1+SUMPRODUCT(MAX(ROW(E4:E$259)*(E262=E4:E$259)))))</f>
@@ -12911,11 +12905,13 @@
         <f aca="false">IF(OR(E262="",E262="!!!",F262="NEW"),"",INDEX(J$1:J261,SUMPRODUCT(MAX(ROW(E$1:E261)*(E262=E$1:E261)))))</f>
         <v/>
       </c>
-      <c r="L262" s="27"/>
+      <c r="L262" s="27" t="s">
+        <v>462</v>
+      </c>
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="21" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E263" s="22" t="str">
         <f aca="false">IF(D263="?OLD","!!!","")</f>
@@ -12990,7 +12986,7 @@
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="21" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E265" s="22" t="str">
         <f aca="false">IF(D265="?OLD","!!!","")</f>
@@ -13024,7 +13020,7 @@
     </row>
     <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="21" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B266" s="28" t="s">
         <v>296</v>
@@ -13036,7 +13032,7 @@
         <v>232</v>
       </c>
       <c r="E266" s="22" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F266" s="23" t="str">
         <f aca="false">IF(OR(E266="",E266="!!!"),"",IF(NOT(ISNA(VLOOKUP(E266,E$1:E265,1,FALSE()))),"OLD",IF(AND(E266&lt;&gt;"",E266&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13062,7 +13058,7 @@
         <v/>
       </c>
       <c r="L266" s="29" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13101,7 +13097,7 @@
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="21" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E268" s="22" t="str">
         <f aca="false">IF(D268="?OLD","!!!","")</f>
@@ -13135,7 +13131,7 @@
     </row>
     <row r="269" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="21" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B269" s="28" t="s">
         <v>230</v>
@@ -13144,7 +13140,7 @@
         <v>237</v>
       </c>
       <c r="E269" s="22" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F269" s="23" t="str">
         <f aca="false">IF(OR(E269="",E269="!!!"),"",IF(NOT(ISNA(VLOOKUP(E269,E$1:E268,1,FALSE()))),"OLD",IF(AND(E269&lt;&gt;"",E269&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13170,7 +13166,7 @@
         <v/>
       </c>
       <c r="L269" s="29" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13209,7 +13205,7 @@
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="21" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E271" s="22" t="str">
         <f aca="false">IF(D271="?OLD","!!!","")</f>
@@ -13277,7 +13273,7 @@
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="21" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E273" s="22" t="str">
         <f aca="false">IF(D273="?OLD","!!!","")</f>
@@ -13311,7 +13307,7 @@
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="21" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B274" s="28" t="s">
         <v>236</v>
@@ -13320,7 +13316,7 @@
         <v>237</v>
       </c>
       <c r="E274" s="22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F274" s="23" t="str">
         <f aca="false">IF(OR(E274="",E274="!!!"),"",IF(NOT(ISNA(VLOOKUP(E274,E$1:E273,1,FALSE()))),"OLD",IF(AND(E274&lt;&gt;"",E274&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13346,7 +13342,7 @@
         <v/>
       </c>
       <c r="L274" s="29" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13388,7 +13384,7 @@
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="21" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13459,9 +13455,9 @@
       </c>
       <c r="L279" s="27"/>
     </row>
-    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="21" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B280" s="28" t="s">
         <v>230</v>
@@ -13473,17 +13469,16 @@
         <v>232</v>
       </c>
       <c r="E280" s="22" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F280" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G280" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H280" s="25" t="str">
-        <f aca="false">IF(J280&lt;&gt;1,"",IF(I280="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H280" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I280" s="26" t="e">
         <f aca="false">IF(OR(E280="",E280="!!!",F280="NEW"),"",INDEX(B4:B$277,-1+SUMPRODUCT(MAX(ROW(E4:E$277)*(E280=E4:E$277)))))</f>
@@ -13498,7 +13493,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L280" s="29" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13577,7 +13572,7 @@
     </row>
     <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="21" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E283" s="22" t="str">
         <f aca="false">IF(D283="?OLD","!!!","")</f>
@@ -13611,7 +13606,7 @@
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="21" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B284" s="28" t="s">
         <v>230</v>
@@ -13683,9 +13678,9 @@
       </c>
       <c r="L285" s="27"/>
     </row>
-    <row r="286" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="21" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B286" s="28" t="s">
         <v>236</v>
@@ -13694,7 +13689,7 @@
         <v>237</v>
       </c>
       <c r="E286" s="22" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F286" s="23" t="str">
         <f aca="false">IF(OR(E286="",E286="!!!"),"",IF(NOT(ISNA(VLOOKUP(E286,E$1:E285,1,FALSE()))),"OLD",IF(AND(E286&lt;&gt;"",E286&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13720,7 +13715,7 @@
         <v/>
       </c>
       <c r="L286" s="29" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13793,7 +13788,7 @@
     </row>
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="21" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E289" s="22" t="str">
         <f aca="false">IF(D289="?OLD","!!!","")</f>
@@ -13873,7 +13868,7 @@
         <v>232</v>
       </c>
       <c r="E291" s="22" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F291" s="23" t="str">
         <f aca="false">IF(OR(E291="",E291="!!!"),"",IF(NOT(ISNA(VLOOKUP(E291,E$1:E290,1,FALSE()))),"OLD",IF(AND(E291&lt;&gt;"",E291&lt;&gt;"!!!"),"NEW","")))</f>
@@ -13914,7 +13909,7 @@
         <v>232</v>
       </c>
       <c r="E292" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F292" s="23" t="s">
         <v>435</v>
@@ -13937,7 +13932,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L292" s="29" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13976,7 +13971,7 @@
     </row>
     <row r="294" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="21" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B294" s="28" t="s">
         <v>270</v>
@@ -13988,10 +13983,10 @@
         <v>232</v>
       </c>
       <c r="E294" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F294" s="23" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="G294" s="24" t="s">
         <v>233</v>
@@ -14013,12 +14008,12 @@
         <v/>
       </c>
       <c r="L294" s="29" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="21" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E295" s="22" t="str">
         <f aca="false">IF(D295="?OLD","!!!","")</f>
@@ -14052,7 +14047,7 @@
     </row>
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="21" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E296" s="22" t="str">
         <f aca="false">IF(D296="?OLD","!!!","")</f>
@@ -14154,7 +14149,7 @@
     </row>
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="21" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B299" s="28" t="s">
         <v>270</v>
@@ -14166,7 +14161,7 @@
         <v>232</v>
       </c>
       <c r="E299" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F299" s="23" t="s">
         <v>435</v>
@@ -14226,7 +14221,7 @@
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="21" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E301" s="22" t="str">
         <f aca="false">IF(D301="?OLD","!!!","")</f>
@@ -14260,7 +14255,7 @@
     </row>
     <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="21" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E302" s="22" t="str">
         <f aca="false">IF(D302="?OLD","!!!","")</f>
@@ -14294,7 +14289,7 @@
     </row>
     <row r="303" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="21" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B303" s="28" t="s">
         <v>342</v>
@@ -14306,7 +14301,7 @@
         <v>232</v>
       </c>
       <c r="E303" s="22" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F303" s="23" t="str">
         <f aca="false">IF(OR(E303="",E303="!!!"),"",IF(NOT(ISNA(VLOOKUP(E303,E$1:E302,1,FALSE()))),"OLD",IF(AND(E303&lt;&gt;"",E303&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14332,7 +14327,7 @@
         <v/>
       </c>
       <c r="L303" s="29" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14371,7 +14366,7 @@
     </row>
     <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="21" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E305" s="22" t="str">
         <f aca="false">IF(D305="?OLD","!!!","")</f>
@@ -14405,7 +14400,7 @@
     </row>
     <row r="306" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="21" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B306" s="28" t="s">
         <v>350</v>
@@ -14417,7 +14412,7 @@
         <v>232</v>
       </c>
       <c r="E306" s="22" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F306" s="23" t="str">
         <f aca="false">IF(OR(E306="",E306="!!!"),"",IF(NOT(ISNA(VLOOKUP(E306,E$1:E305,1,FALSE()))),"OLD",IF(AND(E306&lt;&gt;"",E306&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14443,7 +14438,7 @@
         <v/>
       </c>
       <c r="L306" s="29" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14485,7 +14480,7 @@
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="21" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14524,7 +14519,7 @@
     </row>
     <row r="311" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="21" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B311" s="28" t="s">
         <v>243</v>
@@ -14536,7 +14531,7 @@
         <v>232</v>
       </c>
       <c r="E311" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F311" s="23" t="str">
         <f aca="false">IF(OR(E311="",E311="!!!"),"",IF(NOT(ISNA(VLOOKUP(E311,E$1:E310,1,FALSE()))),"OLD",IF(AND(E311&lt;&gt;"",E311&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14545,9 +14540,8 @@
       <c r="G311" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H311" s="25" t="str">
-        <f aca="false">IF(J311&lt;&gt;1,"",IF(I311="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H311" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I311" s="26" t="str">
         <f aca="false">IF(OR(E311="",E311="!!!",F311="NEW"),"",INDEX(B3:B$309,-1+SUMPRODUCT(MAX(ROW(E3:E$309)*(E311=E3:E$309)))))</f>
@@ -14562,7 +14556,7 @@
         <v>0</v>
       </c>
       <c r="L311" s="29" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="312" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14570,7 +14564,7 @@
         <v>444</v>
       </c>
       <c r="E312" s="22" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F312" s="23"/>
       <c r="G312" s="24"/>
@@ -14591,12 +14585,12 @@
         <v>#VALUE!</v>
       </c>
       <c r="L312" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="21" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E313" s="22" t="str">
         <f aca="false">IF(D313="?OLD","!!!","")</f>
@@ -14738,7 +14732,7 @@
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="21" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E317" s="22" t="str">
         <f aca="false">IF(D317="?OLD","!!!","")</f>
@@ -14849,12 +14843,12 @@
     </row>
     <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="21" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="21" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E322" s="22" t="str">
         <f aca="false">IF(D322="?OLD","!!!","")</f>
@@ -14900,7 +14894,7 @@
         <v>232</v>
       </c>
       <c r="E323" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F323" s="23" t="str">
         <f aca="false">IF(OR(E323="",E323="!!!"),"",IF(NOT(ISNA(VLOOKUP(E323,E$1:E322,1,FALSE()))),"OLD",IF(AND(E323&lt;&gt;"",E323&lt;&gt;"!!!"),"NEW","")))</f>
@@ -14909,9 +14903,8 @@
       <c r="G323" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H323" s="25" t="str">
-        <f aca="false">IF(J323&lt;&gt;1,"",IF(I323="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H323" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I323" s="26" t="str">
         <f aca="false">IF(OR(E323="",E323="!!!",F323="NEW"),"",INDEX(B3:B$321,-1+SUMPRODUCT(MAX(ROW(E3:E$321)*(E323=E3:E$321)))))</f>
@@ -14965,7 +14958,7 @@
     </row>
     <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A325" s="21" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E325" s="22" t="str">
         <f aca="false">IF(D325="?OLD","!!!","")</f>
@@ -14999,10 +14992,10 @@
     </row>
     <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="21" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E326" s="22" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F326" s="23"/>
       <c r="G326" s="24"/>
@@ -15060,7 +15053,7 @@
     </row>
     <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="21" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B328" s="28" t="s">
         <v>230</v>
@@ -15134,7 +15127,7 @@
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A330" s="21" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B330" s="28" t="s">
         <v>236</v>
@@ -15208,7 +15201,7 @@
     </row>
     <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A332" s="21" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B332" s="28" t="s">
         <v>236</v>
@@ -15248,7 +15241,7 @@
     </row>
     <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A333" s="21" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E333" s="22" t="str">
         <f aca="false">IF(D333="?OLD","!!!","")</f>
@@ -15282,7 +15275,7 @@
     </row>
     <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="21" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E334" s="22" t="str">
         <f aca="false">IF(D334="?OLD","!!!","")</f>
@@ -15394,7 +15387,7 @@
     </row>
     <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="21" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15433,7 +15426,7 @@
     </row>
     <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="21" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E340" s="22" t="str">
         <f aca="false">IF(D340="?OLD","!!!","")</f>
@@ -15467,7 +15460,7 @@
     </row>
     <row r="341" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="21" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B341" s="28" t="s">
         <v>243</v>
@@ -15479,7 +15472,7 @@
         <v>232</v>
       </c>
       <c r="E341" s="22" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F341" s="23" t="str">
         <f aca="false">IF(OR(E341="",E341="!!!"),"",IF(NOT(ISNA(VLOOKUP(E341,E$1:E340,1,FALSE()))),"OLD",IF(AND(E341&lt;&gt;"",E341&lt;&gt;"!!!"),"NEW","")))</f>
@@ -15505,12 +15498,12 @@
         <v>0</v>
       </c>
       <c r="L341" s="29" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="21" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E342" s="22" t="str">
         <f aca="false">IF(D342="?OLD","!!!","")</f>
@@ -15544,7 +15537,7 @@
     </row>
     <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E343" s="22" t="str">
         <f aca="false">IF(D343="?OLD","!!!","")</f>
@@ -15578,7 +15571,7 @@
     </row>
     <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="21" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E344" s="22" t="str">
         <f aca="false">IF(D344="?OLD","!!!","")</f>
@@ -15612,7 +15605,7 @@
     </row>
     <row r="345" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="21" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B345" s="28" t="s">
         <v>243</v>
@@ -15621,7 +15614,7 @@
         <v>237</v>
       </c>
       <c r="E345" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F345" s="23" t="str">
         <f aca="false">IF(OR(E345="",E345="!!!"),"",IF(NOT(ISNA(VLOOKUP(E345,E$1:E344,1,FALSE()))),"OLD",IF(AND(E345&lt;&gt;"",E345&lt;&gt;"!!!"),"NEW","")))</f>
@@ -15630,9 +15623,8 @@
       <c r="G345" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H345" s="25" t="str">
-        <f aca="false">IF(J345&lt;&gt;1,"",IF(I345="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H345" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I345" s="26" t="str">
         <f aca="false">IF(OR(E345="",E345="!!!",F345="NEW"),"",INDEX(B8:B$338,-1+SUMPRODUCT(MAX(ROW(E8:E$338)*(E345=E8:E$338)))))</f>
@@ -15647,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="L345" s="29" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15720,7 +15712,7 @@
     </row>
     <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A348" s="21" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E348" s="22" t="str">
         <f aca="false">IF(D348="?OLD","!!!","")</f>
@@ -15788,7 +15780,7 @@
     </row>
     <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A350" s="21" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E350" s="22" t="str">
         <f aca="false">IF(D350="?OLD","!!!","")</f>
@@ -15822,7 +15814,7 @@
     </row>
     <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A351" s="21" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E351" s="22" t="str">
         <f aca="false">IF(D351="?OLD","!!!","")</f>
@@ -15856,7 +15848,7 @@
     </row>
     <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A352" s="21" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B352" s="28" t="s">
         <v>258</v>
@@ -15998,7 +15990,7 @@
     </row>
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="21" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E356" s="22" t="str">
         <f aca="false">IF(D356="?OLD","!!!","")</f>
@@ -16032,7 +16024,7 @@
     </row>
     <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="21" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E357" s="22" t="str">
         <f aca="false">IF(D357="?OLD","!!!","")</f>
@@ -16066,7 +16058,7 @@
     </row>
     <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="21" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E358" s="22" t="str">
         <f aca="false">IF(D358="?OLD","!!!","")</f>
@@ -16171,7 +16163,7 @@
         <v/>
       </c>
       <c r="L360" s="29" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16245,7 +16237,7 @@
         <v>0</v>
       </c>
       <c r="L362" s="29" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16287,7 +16279,7 @@
     </row>
     <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="21" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16326,7 +16318,7 @@
     </row>
     <row r="367" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="21" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B367" s="28" t="s">
         <v>243</v>
@@ -16338,7 +16330,7 @@
         <v>232</v>
       </c>
       <c r="E367" s="22" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F367" s="23" t="s">
         <v>451</v>
@@ -16361,7 +16353,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L367" s="29" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16400,7 +16392,7 @@
     </row>
     <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A369" s="21" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B369" s="28" t="s">
         <v>236</v>
@@ -16474,7 +16466,7 @@
     </row>
     <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="21" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E371" s="22" t="str">
         <f aca="false">IF(D371="?OLD","!!!","")</f>
@@ -16508,7 +16500,7 @@
     </row>
     <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="21" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B372" s="28" t="s">
         <v>236</v>
@@ -16548,7 +16540,7 @@
     </row>
     <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="21" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E373" s="22" t="str">
         <f aca="false">IF(D373="?OLD","!!!","")</f>
@@ -16650,7 +16642,7 @@
     </row>
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="21" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E376" s="22" t="str">
         <f aca="false">IF(D376="?OLD","!!!","")</f>
@@ -16718,7 +16710,7 @@
     </row>
     <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="21" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B378" s="28" t="s">
         <v>230</v>
@@ -16730,7 +16722,7 @@
         <v>232</v>
       </c>
       <c r="E378" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F378" s="23" t="str">
         <f aca="false">IF(OR(E378="",E378="!!!"),"",IF(NOT(ISNA(VLOOKUP(E378,E$1:E377,1,FALSE()))),"OLD",IF(AND(E378&lt;&gt;"",E378&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16739,9 +16731,8 @@
       <c r="G378" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H378" s="25" t="str">
-        <f aca="false">IF(J378&lt;&gt;1,"",IF(I378="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H378" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I378" s="26" t="str">
         <f aca="false">IF(OR(E378="",E378="!!!",F378="NEW"),"",INDEX(B14:B$365,-1+SUMPRODUCT(MAX(ROW(E14:E$365)*(E378=E14:E$365)))))</f>
@@ -16756,7 +16747,7 @@
         <v>0</v>
       </c>
       <c r="L378" s="29" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16798,12 +16789,12 @@
     </row>
     <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="21" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="21" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E382" s="22" t="str">
         <f aca="false">IF(D382="?OLD","!!!","")</f>
@@ -16905,7 +16896,7 @@
     </row>
     <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="21" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B385" s="28" t="s">
         <v>280</v>
@@ -16917,7 +16908,7 @@
         <v>232</v>
       </c>
       <c r="E385" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F385" s="23" t="str">
         <f aca="false">IF(OR(E385="",E385="!!!"),"",IF(NOT(ISNA(VLOOKUP(E385,E$1:E384,1,FALSE()))),"OLD",IF(AND(E385&lt;&gt;"",E385&lt;&gt;"!!!"),"NEW","")))</f>
@@ -16926,9 +16917,8 @@
       <c r="G385" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H385" s="25" t="str">
-        <f aca="false">IF(J385&lt;&gt;1,"",IF(I385="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H385" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I385" s="26" t="str">
         <f aca="false">IF(OR(E385="",E385="!!!",F385="NEW"),"",INDEX(B5:B$381,-1+SUMPRODUCT(MAX(ROW(E5:E$381)*(E385=E5:E$381)))))</f>
@@ -16943,12 +16933,12 @@
         <v>0</v>
       </c>
       <c r="L385" s="29" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="21" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="E386" s="22" t="str">
         <f aca="false">IF(D386="?OLD","!!!","")</f>
@@ -17016,7 +17006,7 @@
     </row>
     <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="21" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E388" s="22" t="str">
         <f aca="false">IF(D388="?OLD","!!!","")</f>
@@ -17084,7 +17074,7 @@
     </row>
     <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="21" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B390" s="28" t="s">
         <v>286</v>
@@ -17096,7 +17086,7 @@
         <v>232</v>
       </c>
       <c r="E390" s="22" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F390" s="23" t="s">
         <v>451</v>
@@ -17191,7 +17181,7 @@
         <v>0</v>
       </c>
       <c r="L392" s="29" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17301,12 +17291,12 @@
         <v/>
       </c>
       <c r="L395" s="29" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="21" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E396" s="22" t="str">
         <f aca="false">IF(D396="?OLD","!!!","")</f>
@@ -17340,7 +17330,7 @@
     </row>
     <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="21" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B397" s="28" t="s">
         <v>270</v>
@@ -17426,7 +17416,7 @@
         <v>232</v>
       </c>
       <c r="E399" s="22" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F399" s="23" t="str">
         <f aca="false">IF(OR(E399="",E399="!!!"),"",IF(NOT(ISNA(VLOOKUP(E399,E$1:E398,1,FALSE()))),"OLD",IF(AND(E399&lt;&gt;"",E399&lt;&gt;"!!!"),"NEW","")))</f>
@@ -17452,7 +17442,7 @@
         <v/>
       </c>
       <c r="L399" s="29" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17491,7 +17481,7 @@
     </row>
     <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A401" s="21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E401" s="22" t="str">
         <f aca="false">IF(D401="?OLD","!!!","")</f>
@@ -17560,12 +17550,12 @@
         <v>0</v>
       </c>
       <c r="L402" s="29" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="21" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E403" s="22" t="str">
         <f aca="false">IF(D403="?OLD","!!!","")</f>
@@ -17599,10 +17589,10 @@
     </row>
     <row r="404" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="21" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="E404" s="22" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="F404" s="23"/>
       <c r="G404" s="24"/>
@@ -17623,7 +17613,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L404" s="29" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17674,7 +17664,7 @@
         <v>232</v>
       </c>
       <c r="E406" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F406" s="23" t="str">
         <f aca="false">IF(OR(E406="",E406="!!!"),"",IF(NOT(ISNA(VLOOKUP(E406,E$1:E405,1,FALSE()))),"OLD",IF(AND(E406&lt;&gt;"",E406&lt;&gt;"!!!"),"NEW","")))</f>
@@ -17700,7 +17690,7 @@
         <v>0</v>
       </c>
       <c r="L406" s="29" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17739,7 +17729,7 @@
     </row>
     <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A408" s="21" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B408" s="28" t="s">
         <v>236</v>
@@ -17813,7 +17803,7 @@
     </row>
     <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="21" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E410" s="22" t="str">
         <f aca="false">IF(D410="?OLD","!!!","")</f>
@@ -17847,7 +17837,7 @@
     </row>
     <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="21" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E411" s="22" t="str">
         <f aca="false">IF(D411="?OLD","!!!","")</f>
@@ -17881,7 +17871,7 @@
     </row>
     <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="21" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B412" s="28" t="s">
         <v>270</v>
@@ -17958,7 +17948,7 @@
     </row>
     <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="21" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17997,7 +17987,7 @@
     </row>
     <row r="417" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="21" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B417" s="28" t="s">
         <v>243</v>
@@ -18009,7 +17999,7 @@
         <v>232</v>
       </c>
       <c r="E417" s="22" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="F417" s="23" t="str">
         <f aca="false">IF(OR(E417="",E417="!!!"),"",IF(NOT(ISNA(VLOOKUP(E417,E$1:E416,1,FALSE()))),"OLD",IF(AND(E417&lt;&gt;"",E417&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18035,12 +18025,12 @@
         <v>0</v>
       </c>
       <c r="L417" s="29" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="21" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E418" s="22" t="str">
         <f aca="false">IF(D418="?OLD","!!!","")</f>
@@ -18074,7 +18064,7 @@
     </row>
     <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="21" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E419" s="22" t="str">
         <f aca="false">IF(D419="?OLD","!!!","")</f>
@@ -18108,7 +18098,7 @@
     </row>
     <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="21" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E420" s="22" t="str">
         <f aca="false">IF(D420="?OLD","!!!","")</f>
@@ -18142,7 +18132,7 @@
     </row>
     <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E421" s="22" t="str">
         <f aca="false">IF(D421="?OLD","!!!","")</f>
@@ -18222,7 +18212,7 @@
         <v>232</v>
       </c>
       <c r="E423" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F423" s="23" t="str">
         <f aca="false">IF(OR(E423="",E423="!!!"),"",IF(NOT(ISNA(VLOOKUP(E423,E$1:E422,1,FALSE()))),"OLD",IF(AND(E423&lt;&gt;"",E423&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18231,9 +18221,8 @@
       <c r="G423" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H423" s="25" t="str">
-        <f aca="false">IF(J423&lt;&gt;1,"",IF(I423="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H423" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I423" s="26" t="n">
         <f aca="false">IF(OR(E423="",E423="!!!",F423="NEW"),"",INDEX(B9:B$415,-1+SUMPRODUCT(MAX(ROW(E9:E$415)*(E423=E9:E$415)))))</f>
@@ -18248,12 +18237,12 @@
         <v>0</v>
       </c>
       <c r="L423" s="29" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="21" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E424" s="22" t="str">
         <f aca="false">IF(D424="?OLD","!!!","")</f>
@@ -18390,7 +18379,7 @@
         <v>0</v>
       </c>
       <c r="L427" s="29" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18429,7 +18418,7 @@
     </row>
     <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="21" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B429" s="28" t="s">
         <v>236</v>
@@ -18441,7 +18430,7 @@
         <v>232</v>
       </c>
       <c r="E429" s="22" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="F429" s="23" t="str">
         <f aca="false">IF(OR(E429="",E429="!!!"),"",IF(NOT(ISNA(VLOOKUP(E429,E$1:E428,1,FALSE()))),"OLD",IF(AND(E429&lt;&gt;"",E429&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18470,7 +18459,7 @@
     </row>
     <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="21" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E430" s="22" t="str">
         <f aca="false">IF(D430="?OLD","!!!","")</f>
@@ -18504,7 +18493,7 @@
     </row>
     <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="21" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B431" s="28" t="s">
         <v>236</v>
@@ -18516,7 +18505,7 @@
         <v>232</v>
       </c>
       <c r="E431" s="22" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="F431" s="23" t="str">
         <f aca="false">IF(OR(E431="",E431="!!!"),"",IF(NOT(ISNA(VLOOKUP(E431,E$1:E430,1,FALSE()))),"OLD",IF(AND(E431&lt;&gt;"",E431&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18613,7 +18602,7 @@
     </row>
     <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="21" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B434" s="28" t="s">
         <v>270</v>
@@ -18625,7 +18614,7 @@
         <v>232</v>
       </c>
       <c r="E434" s="22" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F434" s="23" t="str">
         <f aca="false">IF(OR(E434="",E434="!!!"),"",IF(NOT(ISNA(VLOOKUP(E434,E$1:E433,1,FALSE()))),"OLD",IF(AND(E434&lt;&gt;"",E434&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18691,12 +18680,12 @@
     </row>
     <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="21" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="438" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="21" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B438" s="28" t="s">
         <v>243</v>
@@ -18708,7 +18697,7 @@
         <v>232</v>
       </c>
       <c r="E438" s="22" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="F438" s="23" t="str">
         <f aca="false">IF(OR(E438="",E438="!!!"),"",IF(NOT(ISNA(VLOOKUP(E438,E$1:E437,1,FALSE()))),"OLD",IF(AND(E438&lt;&gt;"",E438&lt;&gt;"!!!"),"NEW","")))</f>
@@ -18734,7 +18723,7 @@
         <v/>
       </c>
       <c r="L438" s="29" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18807,7 +18796,7 @@
     </row>
     <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="21" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E441" s="22" t="str">
         <f aca="false">IF(D441="?OLD","!!!","")</f>
@@ -18841,7 +18830,7 @@
     </row>
     <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="21" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B442" s="28" t="s">
         <v>296</v>
@@ -18949,7 +18938,7 @@
     </row>
     <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="21" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="E445" s="22" t="str">
         <f aca="false">IF(D445="?OLD","!!!","")</f>
@@ -18983,22 +18972,22 @@
     </row>
     <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="21" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B446" s="28" t="s">
         <v>236</v>
       </c>
       <c r="C446" s="28" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D446" s="28" t="s">
         <v>232</v>
       </c>
       <c r="E446" s="22" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F446" s="23" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="G446" s="24"/>
       <c r="H446" s="25" t="str">
@@ -19058,12 +19047,12 @@
     </row>
     <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="21" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
     </row>
     <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="21" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B450" s="28" t="s">
         <v>243</v>
@@ -19075,7 +19064,7 @@
         <v>232</v>
       </c>
       <c r="E450" s="22" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="F450" s="23" t="str">
         <f aca="false">IF(OR(E450="",E450="!!!"),"",IF(NOT(ISNA(VLOOKUP(E450,E$1:E449,1,FALSE()))),"OLD",IF(AND(E450&lt;&gt;"",E450&lt;&gt;"!!!"),"NEW","")))</f>
@@ -19084,9 +19073,8 @@
       <c r="G450" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H450" s="25" t="str">
-        <f aca="false">IF(J450&lt;&gt;1,"",IF(I450="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H450" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I450" s="26" t="str">
         <f aca="false">IF(OR(E450="",E450="!!!",F450="NEW"),"",INDEX(B2:B$449,-1+SUMPRODUCT(MAX(ROW(E2:E$449)*(E450=E2:E$449)))))</f>
@@ -19106,7 +19094,7 @@
     </row>
     <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="21" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E451" s="22" t="str">
         <f aca="false">IF(D451="?OLD","!!!","")</f>
@@ -19140,7 +19128,7 @@
     </row>
     <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="21" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B452" s="28" t="s">
         <v>296</v>
@@ -19214,7 +19202,7 @@
     </row>
     <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="21" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E454" s="22" t="str">
         <f aca="false">IF(D454="?OLD","!!!","")</f>
@@ -19282,7 +19270,7 @@
     </row>
     <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="21" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B456" s="28" t="s">
         <v>236</v>
@@ -19356,7 +19344,7 @@
     </row>
     <row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="21" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B458" s="28" t="s">
         <v>270</v>
@@ -19430,7 +19418,7 @@
     </row>
     <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="21" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E460" s="22" t="str">
         <f aca="false">IF(D460="?OLD","!!!","")</f>
@@ -19473,7 +19461,7 @@
         <v>237</v>
       </c>
       <c r="E461" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F461" s="23" t="str">
         <f aca="false">IF(OR(E461="",E461="!!!"),"",IF(NOT(ISNA(VLOOKUP(E461,E$1:E460,1,FALSE()))),"OLD",IF(AND(E461&lt;&gt;"",E461&lt;&gt;"!!!"),"NEW","")))</f>
@@ -19499,12 +19487,12 @@
         <v>0</v>
       </c>
       <c r="L461" s="29" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="21" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E462" s="22" t="str">
         <f aca="false">IF(D462="?OLD","!!!","")</f>
@@ -19538,7 +19526,7 @@
     </row>
     <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="21" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E463" s="22" t="str">
         <f aca="false">IF(D463="?OLD","!!!","")</f>
@@ -19572,7 +19560,7 @@
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="21" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E464" s="22" t="str">
         <f aca="false">IF(D464="?OLD","!!!","")</f>
@@ -19606,7 +19594,7 @@
     </row>
     <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="21" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E465" s="22" t="str">
         <f aca="false">IF(D465="?OLD","!!!","")</f>
@@ -19640,7 +19628,7 @@
     </row>
     <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="21" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="E466" s="22" t="str">
         <f aca="false">IF(D466="?OLD","!!!","")</f>
@@ -19674,7 +19662,7 @@
     </row>
     <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="21" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E467" s="22" t="str">
         <f aca="false">IF(D467="?OLD","!!!","")</f>
@@ -19785,12 +19773,12 @@
     </row>
     <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A471" s="21" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
     </row>
     <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="21" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E472" s="22" t="str">
         <f aca="false">IF(D472="?OLD","!!!","")</f>
@@ -19858,7 +19846,7 @@
     </row>
     <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="21" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E474" s="22" t="str">
         <f aca="false">IF(D474="?OLD","!!!","")</f>
@@ -19930,7 +19918,7 @@
         <v>0</v>
       </c>
       <c r="L475" s="29" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19941,7 +19929,7 @@
         <v>280</v>
       </c>
       <c r="C476" s="28" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D476" s="28" t="s">
         <v>232</v>
@@ -19972,12 +19960,12 @@
         <v/>
       </c>
       <c r="L476" s="29" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
     </row>
     <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="21" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E477" s="22" t="str">
         <f aca="false">IF(D477="?OLD","!!!","")</f>
@@ -20011,7 +19999,7 @@
     </row>
     <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="21" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E478" s="22" t="str">
         <f aca="false">IF(D478="?OLD","!!!","")</f>
@@ -20045,7 +20033,7 @@
     </row>
     <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="21" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E479" s="22" t="str">
         <f aca="false">IF(D479="?OLD","!!!","")</f>
@@ -20082,13 +20070,13 @@
         <v>368</v>
       </c>
       <c r="B480" s="28" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C480" s="28" t="s">
         <v>311</v>
       </c>
       <c r="E480" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F480" s="23" t="str">
         <f aca="false">IF(OR(E480="",E480="!!!"),"",IF(NOT(ISNA(VLOOKUP(E480,E$1:E479,1,FALSE()))),"OLD",IF(AND(E480&lt;&gt;"",E480&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20097,9 +20085,8 @@
       <c r="G480" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H480" s="25" t="str">
-        <f aca="false">IF(J480&lt;&gt;1,"",IF(I480="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H480" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I480" s="26" t="n">
         <f aca="false">IF(OR(E480="",E480="!!!",F480="NEW"),"",INDEX(B10:B$471,-1+SUMPRODUCT(MAX(ROW(E10:E$471)*(E480=E10:E$471)))))</f>
@@ -20114,7 +20101,7 @@
         <v>0</v>
       </c>
       <c r="L480" s="29" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
     </row>
     <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20153,7 +20140,7 @@
     </row>
     <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A482" s="21" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B482" s="28" t="s">
         <v>236</v>
@@ -20259,9 +20246,9 @@
       </c>
       <c r="L484" s="27"/>
     </row>
-    <row r="485" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="485" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A485" s="21" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B485" s="28" t="s">
         <v>243</v>
@@ -20273,7 +20260,7 @@
         <v>232</v>
       </c>
       <c r="E485" s="22" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F485" s="23" t="str">
         <f aca="false">IF(OR(E485="",E485="!!!"),"",IF(NOT(ISNA(VLOOKUP(E485,E$1:E484,1,FALSE()))),"OLD",IF(AND(E485&lt;&gt;"",E485&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20299,12 +20286,12 @@
         <v/>
       </c>
       <c r="L485" s="29" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
     </row>
     <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A486" s="21" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E486" s="22" t="str">
         <f aca="false">IF(D486="?OLD","!!!","")</f>
@@ -20350,7 +20337,7 @@
         <v>232</v>
       </c>
       <c r="E487" s="22" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F487" s="23" t="str">
         <f aca="false">IF(OR(E487="",E487="!!!"),"",IF(NOT(ISNA(VLOOKUP(E487,E$1:E486,1,FALSE()))),"OLD",IF(AND(E487&lt;&gt;"",E487&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20379,7 +20366,7 @@
     </row>
     <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A488" s="21" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E488" s="22" t="str">
         <f aca="false">IF(D488="?OLD","!!!","")</f>
@@ -20413,7 +20400,7 @@
     </row>
     <row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A489" s="21" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E489" s="22" t="str">
         <f aca="false">IF(D489="?OLD","!!!","")</f>
@@ -20459,7 +20446,7 @@
         <v>232</v>
       </c>
       <c r="E490" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F490" s="23" t="str">
         <f aca="false">IF(OR(E490="",E490="!!!"),"",IF(NOT(ISNA(VLOOKUP(E490,E$1:E489,1,FALSE()))),"OLD",IF(AND(E490&lt;&gt;"",E490&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20485,7 +20472,7 @@
         <v/>
       </c>
       <c r="L490" s="29" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20524,12 +20511,12 @@
     </row>
     <row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A493" s="21" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
     </row>
     <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A494" s="21" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E494" s="22" t="str">
         <f aca="false">IF(D494="?OLD","!!!","")</f>
@@ -20609,7 +20596,7 @@
         <v>232</v>
       </c>
       <c r="E496" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F496" s="23" t="str">
         <f aca="false">IF(OR(E496="",E496="!!!"),"",IF(NOT(ISNA(VLOOKUP(E496,E$1:E495,1,FALSE()))),"OLD",IF(AND(E496&lt;&gt;"",E496&lt;&gt;"!!!"),"NEW","")))</f>
@@ -20618,9 +20605,8 @@
       <c r="G496" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H496" s="25" t="str">
-        <f aca="false">IF(J496&lt;&gt;1,"",IF(I496="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H496" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I496" s="26" t="n">
         <f aca="false">IF(OR(E496="",E496="!!!",F496="NEW"),"",INDEX(B4:B$493,-1+SUMPRODUCT(MAX(ROW(E4:E$493)*(E496=E4:E$493)))))</f>
@@ -20638,7 +20624,7 @@
     </row>
     <row r="497" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A497" s="21" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B497" s="28" t="s">
         <v>230</v>
@@ -20650,7 +20636,7 @@
         <v>232</v>
       </c>
       <c r="E497" s="22" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="F497" s="23" t="s">
         <v>451</v>
@@ -20673,7 +20659,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L497" s="29" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20712,7 +20698,7 @@
     </row>
     <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A499" s="21" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E499" s="22" t="str">
         <f aca="false">IF(D499="?OLD","!!!","")</f>
@@ -20746,7 +20732,7 @@
     </row>
     <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A500" s="21" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="E500" s="22" t="str">
         <f aca="false">IF(D500="?OLD","!!!","")</f>
@@ -20780,7 +20766,7 @@
     </row>
     <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A501" s="21" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B501" s="28" t="s">
         <v>286</v>
@@ -20854,7 +20840,7 @@
     </row>
     <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A503" s="21" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E503" s="22" t="str">
         <f aca="false">IF(D503="?OLD","!!!","")</f>
@@ -20888,7 +20874,7 @@
     </row>
     <row r="504" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A504" s="21" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B504" s="28" t="s">
         <v>258</v>
@@ -20996,7 +20982,7 @@
     </row>
     <row r="507" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A507" s="21" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E507" s="22" t="str">
         <f aca="false">IF(D507="?OLD","!!!","")</f>
@@ -21104,7 +21090,7 @@
     </row>
     <row r="510" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A510" s="21" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E510" s="22" t="str">
         <f aca="false">IF(D510="?OLD","!!!","")</f>
@@ -21178,7 +21164,7 @@
     </row>
     <row r="512" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A512" s="21" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E512" s="22" t="str">
         <f aca="false">IF(D512="?OLD","!!!","")</f>
@@ -21212,7 +21198,7 @@
     </row>
     <row r="513" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A513" s="21" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E513" s="22" t="str">
         <f aca="false">IF(D513="?OLD","!!!","")</f>
@@ -21280,7 +21266,7 @@
     </row>
     <row r="515" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A515" s="21" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E515" s="22" t="str">
         <f aca="false">IF(D515="?OLD","!!!","")</f>
@@ -21314,7 +21300,7 @@
     </row>
     <row r="516" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A516" s="21" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E516" s="22" t="str">
         <f aca="false">IF(D516="?OLD","!!!","")</f>
@@ -21348,7 +21334,7 @@
     </row>
     <row r="517" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A517" s="21" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B517" s="28" t="s">
         <v>270</v>
@@ -21425,12 +21411,12 @@
     </row>
     <row r="520" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A520" s="21" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="521" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A521" s="21" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B521" s="28" t="s">
         <v>243</v>
@@ -21442,7 +21428,7 @@
         <v>232</v>
       </c>
       <c r="E521" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F521" s="23" t="str">
         <f aca="false">IF(OR(E521="",E521="!!!"),"",IF(NOT(ISNA(VLOOKUP(E521,E$1:E520,1,FALSE()))),"OLD",IF(AND(E521&lt;&gt;"",E521&lt;&gt;"!!!"),"NEW","")))</f>
@@ -21451,9 +21437,8 @@
       <c r="G521" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H521" s="25" t="str">
-        <f aca="false">IF(J521&lt;&gt;1,"",IF(I521="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H521" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I521" s="26" t="str">
         <f aca="false">IF(OR(E521="",E521="!!!",F521="NEW"),"",INDEX(B2:B$520,-1+SUMPRODUCT(MAX(ROW(E2:E$520)*(E521=E2:E$520)))))</f>
@@ -21468,12 +21453,12 @@
         <v>0</v>
       </c>
       <c r="L521" s="29" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="522" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A522" s="21" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E522" s="22" t="str">
         <f aca="false">IF(D522="?OLD","!!!","")</f>
@@ -21507,7 +21492,7 @@
     </row>
     <row r="523" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A523" s="21" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B523" s="28" t="s">
         <v>296</v>
@@ -21581,7 +21566,7 @@
     </row>
     <row r="525" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A525" s="21" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="B525" s="28" t="s">
         <v>236</v>
@@ -21655,7 +21640,7 @@
     </row>
     <row r="527" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A527" s="21" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B527" s="28" t="s">
         <v>270</v>
@@ -21729,7 +21714,7 @@
     </row>
     <row r="529" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A529" s="21" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B529" s="28" t="s">
         <v>270</v>
@@ -21837,7 +21822,7 @@
     </row>
     <row r="532" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A532" s="21" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="E532" s="22" t="str">
         <f aca="false">IF(D532="?OLD","!!!","")</f>
@@ -21871,7 +21856,7 @@
     </row>
     <row r="533" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A533" s="21" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B533" s="28" t="s">
         <v>230</v>
@@ -21945,7 +21930,7 @@
     </row>
     <row r="535" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A535" s="21" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E535" s="22" t="str">
         <f aca="false">IF(D535="?OLD","!!!","")</f>
@@ -22025,7 +22010,7 @@
         <v>232</v>
       </c>
       <c r="E537" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F537" s="23" t="str">
         <f aca="false">IF(OR(E537="",E537="!!!"),"",IF(NOT(ISNA(VLOOKUP(E537,E$1:E536,1,FALSE()))),"OLD",IF(AND(E537&lt;&gt;"",E537&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22054,7 +22039,7 @@
     </row>
     <row r="538" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A538" s="21" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B538" s="28" t="s">
         <v>270</v>
@@ -22066,7 +22051,7 @@
         <v>232</v>
       </c>
       <c r="E538" s="22" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="F538" s="23" t="str">
         <f aca="false">IF(OR(E538="",E538="!!!"),"",IF(NOT(ISNA(VLOOKUP(E538,E$1:E537,1,FALSE()))),"OLD",IF(AND(E538&lt;&gt;"",E538&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22092,7 +22077,7 @@
         <v/>
       </c>
       <c r="L538" s="29" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="539" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22134,12 +22119,12 @@
     </row>
     <row r="541" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A541" s="21" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
     </row>
     <row r="542" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A542" s="21" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E542" s="22" t="str">
         <f aca="false">IF(D542="?OLD","!!!","")</f>
@@ -22216,7 +22201,7 @@
         <v>237</v>
       </c>
       <c r="E544" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F544" s="23" t="str">
         <f aca="false">IF(OR(E544="",E544="!!!"),"",IF(NOT(ISNA(VLOOKUP(E544,E$1:E543,1,FALSE()))),"OLD",IF(AND(E544&lt;&gt;"",E544&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22225,9 +22210,8 @@
       <c r="G544" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H544" s="25" t="str">
-        <f aca="false">IF(J544&lt;&gt;1,"",IF(I544="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H544" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I544" s="26" t="n">
         <f aca="false">IF(OR(E544="",E544="!!!",F544="NEW"),"",INDEX(B4:B$541,-1+SUMPRODUCT(MAX(ROW(E4:E$541)*(E544=E4:E$541)))))</f>
@@ -22242,12 +22226,12 @@
         <v>0</v>
       </c>
       <c r="L544" s="29" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="545" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A545" s="21" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E545" s="22" t="str">
         <f aca="false">IF(D545="?OLD","!!!","")</f>
@@ -22315,7 +22299,7 @@
     </row>
     <row r="547" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A547" s="21" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B547" s="28" t="s">
         <v>296</v>
@@ -22327,7 +22311,7 @@
         <v>232</v>
       </c>
       <c r="E547" s="22" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F547" s="23" t="str">
         <f aca="false">IF(OR(E547="",E547="!!!"),"",IF(NOT(ISNA(VLOOKUP(E547,E$1:E546,1,FALSE()))),"OLD",IF(AND(E547&lt;&gt;"",E547&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22353,7 +22337,7 @@
         <v/>
       </c>
       <c r="L547" s="29" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="548" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22392,7 +22376,7 @@
     </row>
     <row r="549" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A549" s="21" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E549" s="22" t="str">
         <f aca="false">IF(D549="?OLD","!!!","")</f>
@@ -22426,7 +22410,7 @@
     </row>
     <row r="550" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A550" s="21" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E550" s="22" t="str">
         <f aca="false">IF(D550="?OLD","!!!","")</f>
@@ -22460,7 +22444,7 @@
     </row>
     <row r="551" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A551" s="21" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E551" s="22" t="str">
         <f aca="false">IF(D551="?OLD","!!!","")</f>
@@ -22494,7 +22478,7 @@
     </row>
     <row r="552" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A552" s="21" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B552" s="28" t="s">
         <v>258</v>
@@ -22531,7 +22515,7 @@
         <v/>
       </c>
       <c r="L552" s="29" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
     </row>
     <row r="553" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22570,7 +22554,7 @@
     </row>
     <row r="554" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A554" s="21" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B554" s="28" t="s">
         <v>270</v>
@@ -22647,12 +22631,12 @@
     </row>
     <row r="557" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A557" s="21" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="558" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A558" s="21" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E558" s="22" t="str">
         <f aca="false">IF(D558="?OLD","!!!","")</f>
@@ -22720,7 +22704,7 @@
     </row>
     <row r="560" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A560" s="21" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E560" s="22" t="str">
         <f aca="false">IF(D560="?OLD","!!!","")</f>
@@ -22788,7 +22772,7 @@
     </row>
     <row r="562" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A562" s="21" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E562" s="22" t="str">
         <f aca="false">IF(D562="?OLD","!!!","")</f>
@@ -22908,7 +22892,7 @@
         <v>232</v>
       </c>
       <c r="E565" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F565" s="23" t="str">
         <f aca="false">IF(OR(E565="",E565="!!!"),"",IF(NOT(ISNA(VLOOKUP(E565,E$1:E564,1,FALSE()))),"OLD",IF(AND(E565&lt;&gt;"",E565&lt;&gt;"!!!"),"NEW","")))</f>
@@ -22917,9 +22901,8 @@
       <c r="G565" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H565" s="25" t="str">
-        <f aca="false">IF(J565&lt;&gt;1,"",IF(I565="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H565" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I565" s="26" t="n">
         <f aca="false">IF(OR(E565="",E565="!!!",F565="NEW"),"",INDEX(B9:B$557,-1+SUMPRODUCT(MAX(ROW(E9:E$557)*(E565=E9:E$557)))))</f>
@@ -22937,7 +22920,7 @@
     </row>
     <row r="566" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A566" s="21" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="E566" s="22" t="str">
         <f aca="false">IF(D566="?OLD","!!!","")</f>
@@ -22971,7 +22954,7 @@
     </row>
     <row r="567" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A567" s="21" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="E567" s="22" t="str">
         <f aca="false">IF(D567="?OLD","!!!","")</f>
@@ -23039,7 +23022,7 @@
     </row>
     <row r="569" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A569" s="21" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="E569" s="22" t="str">
         <f aca="false">IF(D569="?OLD","!!!","")</f>
@@ -23107,7 +23090,7 @@
     </row>
     <row r="571" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A571" s="21" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B571" s="28" t="s">
         <v>236</v>
@@ -23181,7 +23164,7 @@
     </row>
     <row r="573" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A573" s="21" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B573" s="28" t="s">
         <v>270</v>
@@ -23258,12 +23241,12 @@
     </row>
     <row r="576" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A576" s="21" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="577" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A577" s="21" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="E577" s="22" t="str">
         <f aca="false">IF(D577="?OLD","!!!","")</f>
@@ -23343,7 +23326,7 @@
         <v>232</v>
       </c>
       <c r="E579" s="22" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="F579" s="23" t="str">
         <f aca="false">IF(OR(E579="",E579="!!!"),"",IF(NOT(ISNA(VLOOKUP(E579,E$1:E578,1,FALSE()))),"OLD",IF(AND(E579&lt;&gt;"",E579&lt;&gt;"!!!"),"NEW","")))</f>
@@ -23369,7 +23352,7 @@
         <v/>
       </c>
       <c r="L579" s="29" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
     </row>
     <row r="580" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23442,16 +23425,16 @@
     </row>
     <row r="582" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A582" s="21" t="s">
-        <v>678</v>
-      </c>
-      <c r="B582" s="30" t="s">
+        <v>679</v>
+      </c>
+      <c r="B582" s="21" t="s">
         <v>236</v>
       </c>
       <c r="C582" s="1" t="s">
         <v>231</v>
       </c>
       <c r="E582" s="22" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F582" s="23" t="str">
         <f aca="false">IF(OR(E582="",E582="!!!"),"",IF(NOT(ISNA(VLOOKUP(E582,E$1:E581,1,FALSE()))),"OLD",IF(AND(E582&lt;&gt;"",E582&lt;&gt;"!!!"),"NEW","")))</f>
@@ -23477,12 +23460,12 @@
         <v/>
       </c>
       <c r="L582" s="29" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
     </row>
     <row r="583" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A583" s="21" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E583" s="22" t="str">
         <f aca="false">IF(D583="?OLD","!!!","")</f>
@@ -23550,7 +23533,7 @@
     </row>
     <row r="585" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A585" s="21" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B585" s="28" t="s">
         <v>236</v>
@@ -23587,12 +23570,12 @@
         <v/>
       </c>
       <c r="L585" s="29" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
     </row>
     <row r="586" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A586" s="21" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E586" s="22" t="str">
         <f aca="false">IF(D586="?OLD","!!!","")</f>
@@ -23626,7 +23609,7 @@
     </row>
     <row r="587" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A587" s="21" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E587" s="22" t="str">
         <f aca="false">IF(D587="?OLD","!!!","")</f>
@@ -23658,9 +23641,9 @@
       </c>
       <c r="L587" s="27"/>
     </row>
-    <row r="588" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="588" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A588" s="21" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B588" s="28" t="s">
         <v>263</v>
@@ -23672,7 +23655,7 @@
         <v>232</v>
       </c>
       <c r="E588" s="22" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F588" s="23" t="str">
         <f aca="false">IF(OR(E588="",E588="!!!"),"",IF(NOT(ISNA(VLOOKUP(E588,E$1:E587,1,FALSE()))),"OLD",IF(AND(E588&lt;&gt;"",E588&lt;&gt;"!!!"),"NEW","")))</f>
@@ -23735,7 +23718,7 @@
     </row>
     <row r="590" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A590" s="21" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B590" s="28" t="s">
         <v>342</v>
@@ -23747,7 +23730,7 @@
         <v>232</v>
       </c>
       <c r="E590" s="22" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="F590" s="23" t="str">
         <f aca="false">IF(OR(E590="",E590="!!!"),"",IF(NOT(ISNA(VLOOKUP(E590,E$1:E589,1,FALSE()))),"OLD",IF(AND(E590&lt;&gt;"",E590&lt;&gt;"!!!"),"NEW","")))</f>
@@ -23773,12 +23756,12 @@
         <v/>
       </c>
       <c r="L590" s="29" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
     </row>
     <row r="591" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A591" s="21" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E591" s="22" t="str">
         <f aca="false">IF(D591="?OLD","!!!","")</f>
@@ -23846,7 +23829,7 @@
     </row>
     <row r="593" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A593" s="21" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B593" s="28" t="s">
         <v>296</v>
@@ -23952,7 +23935,7 @@
     </row>
     <row r="596" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A596" s="21" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="E596" s="22" t="str">
         <f aca="false">IF(D596="?OLD","!!!","")</f>
@@ -23986,7 +23969,7 @@
     </row>
     <row r="597" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A597" s="21" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="E597" s="22" t="str">
         <f aca="false">IF(D597="?OLD","!!!","")</f>
@@ -24020,7 +24003,7 @@
     </row>
     <row r="598" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A598" s="21" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E598" s="22" t="str">
         <f aca="false">IF(D598="?OLD","!!!","")</f>
@@ -24054,7 +24037,7 @@
     </row>
     <row r="599" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A599" s="21" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B599" s="28" t="s">
         <v>236</v>
@@ -24066,7 +24049,7 @@
         <v>232</v>
       </c>
       <c r="E599" s="22" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="F599" s="23" t="str">
         <f aca="false">IF(OR(E599="",E599="!!!"),"",IF(NOT(ISNA(VLOOKUP(E599,E$1:E598,1,FALSE()))),"OLD",IF(AND(E599&lt;&gt;"",E599&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24092,12 +24075,12 @@
         <v/>
       </c>
       <c r="L599" s="29" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
     </row>
     <row r="600" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A600" s="21" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="E600" s="22" t="str">
         <f aca="false">IF(D600="?OLD","!!!","")</f>
@@ -24131,7 +24114,7 @@
     </row>
     <row r="601" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A601" s="21" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B601" s="28" t="s">
         <v>270</v>
@@ -24208,12 +24191,12 @@
     </row>
     <row r="604" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A604" s="21" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
     </row>
     <row r="605" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A605" s="21" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B605" s="28" t="s">
         <v>230</v>
@@ -24389,7 +24372,7 @@
     </row>
     <row r="610" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A610" s="21" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="E610" s="22" t="str">
         <f aca="false">IF(D610="?OLD","!!!","")</f>
@@ -24423,7 +24406,7 @@
     </row>
     <row r="611" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A611" s="21" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B611" s="28" t="s">
         <v>230</v>
@@ -24435,7 +24418,7 @@
         <v>232</v>
       </c>
       <c r="E611" s="22" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="F611" s="23" t="str">
         <f aca="false">IF(OR(E611="",E611="!!!"),"",IF(NOT(ISNA(VLOOKUP(E611,E$1:E610,1,FALSE()))),"OLD",IF(AND(E611&lt;&gt;"",E611&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24461,7 +24444,7 @@
         <v/>
       </c>
       <c r="L611" s="29" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
     </row>
     <row r="612" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24500,7 +24483,7 @@
     </row>
     <row r="613" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A613" s="21" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E613" s="22" t="str">
         <f aca="false">IF(D613="?OLD","!!!","")</f>
@@ -24543,7 +24526,7 @@
         <v>237</v>
       </c>
       <c r="E614" s="22" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F614" s="23" t="str">
         <f aca="false">IF(OR(E614="",E614="!!!"),"",IF(NOT(ISNA(VLOOKUP(E614,E$1:E613,1,FALSE()))),"OLD",IF(AND(E614&lt;&gt;"",E614&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24572,7 +24555,7 @@
     </row>
     <row r="615" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A615" s="21" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E615" s="22" t="str">
         <f aca="false">IF(D615="?OLD","!!!","")</f>
@@ -24606,7 +24589,7 @@
     </row>
     <row r="616" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A616" s="21" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E616" s="22" t="str">
         <f aca="false">IF(D616="?OLD","!!!","")</f>
@@ -24708,7 +24691,7 @@
     </row>
     <row r="619" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A619" s="21" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E619" s="22" t="str">
         <f aca="false">IF(D619="?OLD","!!!","")</f>
@@ -24742,7 +24725,7 @@
     </row>
     <row r="620" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A620" s="21" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B620" s="28" t="s">
         <v>236</v>
@@ -24754,7 +24737,7 @@
         <v>232</v>
       </c>
       <c r="E620" s="22" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="F620" s="23" t="str">
         <f aca="false">IF(OR(E620="",E620="!!!"),"",IF(NOT(ISNA(VLOOKUP(E620,E$1:E619,1,FALSE()))),"OLD",IF(AND(E620&lt;&gt;"",E620&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24780,7 +24763,7 @@
         <v/>
       </c>
       <c r="L620" s="29" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
     </row>
     <row r="621" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24853,7 +24836,7 @@
     </row>
     <row r="623" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A623" s="21" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B623" s="28" t="s">
         <v>236</v>
@@ -24865,7 +24848,7 @@
         <v>232</v>
       </c>
       <c r="E623" s="22" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="F623" s="23" t="str">
         <f aca="false">IF(OR(E623="",E623="!!!"),"",IF(NOT(ISNA(VLOOKUP(E623,E$1:E622,1,FALSE()))),"OLD",IF(AND(E623&lt;&gt;"",E623&lt;&gt;"!!!"),"NEW","")))</f>
@@ -24891,7 +24874,7 @@
         <v/>
       </c>
       <c r="L623" s="29" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
     </row>
     <row r="624" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24930,7 +24913,7 @@
     </row>
     <row r="625" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A625" s="21" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="E625" s="22" t="str">
         <f aca="false">IF(D625="?OLD","!!!","")</f>
@@ -24964,10 +24947,10 @@
     </row>
     <row r="626" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A626" s="21" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B626" s="28" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C626" s="28" t="s">
         <v>237</v>
@@ -25041,12 +25024,12 @@
     </row>
     <row r="629" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A629" s="21" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="630" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A630" s="21" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E630" s="22" t="str">
         <f aca="false">IF(D630="?OLD","!!!","")</f>
@@ -25080,7 +25063,7 @@
     </row>
     <row r="631" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A631" s="21" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E631" s="22" t="str">
         <f aca="false">IF(D631="?OLD","!!!","")</f>
@@ -25148,7 +25131,7 @@
     </row>
     <row r="633" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A633" s="21" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="E633" s="22" t="str">
         <f aca="false">IF(D633="?OLD","!!!","")</f>
@@ -25182,7 +25165,7 @@
     </row>
     <row r="634" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A634" s="21" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B634" s="28" t="s">
         <v>243</v>
@@ -25219,7 +25202,7 @@
         <v/>
       </c>
       <c r="L634" s="29" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
     </row>
     <row r="635" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25258,7 +25241,7 @@
     </row>
     <row r="636" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A636" s="21" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E636" s="22" t="str">
         <f aca="false">IF(D636="?OLD","!!!","")</f>
@@ -25292,7 +25275,7 @@
     </row>
     <row r="637" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A637" s="21" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E637" s="22" t="str">
         <f aca="false">IF(D637="?OLD","!!!","")</f>
@@ -25324,9 +25307,9 @@
       </c>
       <c r="L637" s="27"/>
     </row>
-    <row r="638" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="638" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A638" s="21" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B638" s="28" t="s">
         <v>236</v>
@@ -25335,10 +25318,10 @@
         <v>237</v>
       </c>
       <c r="E638" s="22" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F638" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G638" s="24" t="s">
         <v>370</v>
@@ -25360,7 +25343,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L638" s="29" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
     </row>
     <row r="639" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25399,7 +25382,7 @@
     </row>
     <row r="640" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A640" s="21" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="E640" s="22" t="str">
         <f aca="false">IF(D640="?OLD","!!!","")</f>
@@ -25433,7 +25416,7 @@
     </row>
     <row r="641" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A641" s="21" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E641" s="22" t="str">
         <f aca="false">IF(D641="?OLD","!!!","")</f>
@@ -25535,7 +25518,7 @@
     </row>
     <row r="644" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A644" s="21" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B644" s="28" t="s">
         <v>270</v>
@@ -25547,7 +25530,7 @@
         <v>232</v>
       </c>
       <c r="E644" s="22" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="F644" s="23" t="str">
         <f aca="false">IF(OR(E644="",E644="!!!"),"",IF(NOT(ISNA(VLOOKUP(E644,E$1:E643,1,FALSE()))),"OLD",IF(AND(E644&lt;&gt;"",E644&lt;&gt;"!!!"),"NEW","")))</f>
@@ -25556,9 +25539,8 @@
       <c r="G644" s="24" t="s">
         <v>287</v>
       </c>
-      <c r="H644" s="25" t="str">
-        <f aca="false">IF(J644&lt;&gt;1,"",IF(I644="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H644" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I644" s="26" t="n">
         <f aca="false">IF(OR(E644="",E644="!!!",F644="NEW"),"",INDEX(B16:B$629,-1+SUMPRODUCT(MAX(ROW(E16:E$629)*(E644=E16:E$629)))))</f>
@@ -25572,7 +25554,9 @@
         <f aca="false">IF(OR(E644="",E644="!!!",F644="NEW"),"",INDEX(J$1:J643,SUMPRODUCT(MAX(ROW(E$1:E643)*(E644=E$1:E643)))))</f>
         <v/>
       </c>
-      <c r="L644" s="27"/>
+      <c r="L644" s="27" t="s">
+        <v>728</v>
+      </c>
     </row>
     <row r="645" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A645" s="21" t="s">
@@ -25610,7 +25594,7 @@
     </row>
     <row r="646" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A646" s="21" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="E646" s="22" t="str">
         <f aca="false">IF(D646="?OLD","!!!","")</f>
@@ -25678,7 +25662,7 @@
     </row>
     <row r="648" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A648" s="21" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="E648" s="22" t="str">
         <f aca="false">IF(D648="?OLD","!!!","")</f>
@@ -25712,7 +25696,7 @@
     </row>
     <row r="649" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A649" s="21" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E649" s="22" t="str">
         <f aca="false">IF(D649="?OLD","!!!","")</f>
@@ -25746,7 +25730,7 @@
     </row>
     <row r="650" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A650" s="21" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B650" s="28" t="s">
         <v>236</v>
@@ -25758,7 +25742,7 @@
         <v>232</v>
       </c>
       <c r="E650" s="22" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="F650" s="23" t="str">
         <f aca="false">IF(OR(E650="",E650="!!!"),"",IF(NOT(ISNA(VLOOKUP(E650,E$1:E649,1,FALSE()))),"OLD",IF(AND(E650&lt;&gt;"",E650&lt;&gt;"!!!"),"NEW","")))</f>
@@ -25855,7 +25839,7 @@
     </row>
     <row r="653" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A653" s="21" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E653" s="22" t="str">
         <f aca="false">IF(D653="?OLD","!!!","")</f>
@@ -25889,7 +25873,7 @@
     </row>
     <row r="654" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A654" s="21" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="B654" s="28" t="s">
         <v>286</v>
@@ -25963,7 +25947,7 @@
     </row>
     <row r="656" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A656" s="21" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B656" s="28" t="s">
         <v>263</v>
@@ -25975,7 +25959,7 @@
         <v>232</v>
       </c>
       <c r="E656" s="22" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="F656" s="23" t="str">
         <f aca="false">IF(OR(E656="",E656="!!!"),"",IF(NOT(ISNA(VLOOKUP(E656,E$1:E655,1,FALSE()))),"OLD",IF(AND(E656&lt;&gt;"",E656&lt;&gt;"!!!"),"NEW","")))</f>
@@ -26072,7 +26056,7 @@
     </row>
     <row r="659" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A659" s="21" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B659" s="28" t="s">
         <v>230</v>
@@ -26084,7 +26068,7 @@
         <v>232</v>
       </c>
       <c r="E659" s="22" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F659" s="23" t="str">
         <f aca="false">IF(OR(E659="",E659="!!!"),"",IF(NOT(ISNA(VLOOKUP(E659,E$1:E658,1,FALSE()))),"OLD",IF(AND(E659&lt;&gt;"",E659&lt;&gt;"!!!"),"NEW","")))</f>
@@ -26150,12 +26134,12 @@
     </row>
     <row r="662" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A662" s="21" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="663" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A663" s="21" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B663" s="28" t="s">
         <v>230</v>
@@ -26226,7 +26210,7 @@
     </row>
     <row r="665" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A665" s="21" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="E665" s="22" t="str">
         <f aca="false">IF(D665="?OLD","!!!","")</f>
@@ -26329,7 +26313,7 @@
         <v>0</v>
       </c>
       <c r="L667" s="29" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
     </row>
     <row r="668" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26368,7 +26352,7 @@
     </row>
     <row r="669" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A669" s="21" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="E669" s="22" t="str">
         <f aca="false">IF(D669="?OLD","!!!","")</f>
@@ -26436,7 +26420,7 @@
     </row>
     <row r="671" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A671" s="21" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="E671" s="22" t="str">
         <f aca="false">IF(D671="?OLD","!!!","")</f>
@@ -26504,7 +26488,7 @@
     </row>
     <row r="673" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A673" s="21" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="E673" s="22" t="str">
         <f aca="false">IF(D673="?OLD","!!!","")</f>
@@ -26538,7 +26522,7 @@
     </row>
     <row r="674" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A674" s="21" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B674" s="28" t="s">
         <v>230</v>
@@ -26575,7 +26559,7 @@
         <v/>
       </c>
       <c r="L674" s="29" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
     </row>
     <row r="675" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26648,7 +26632,7 @@
     </row>
     <row r="677" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A677" s="21" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E677" s="22" t="str">
         <f aca="false">IF(D677="?OLD","!!!","")</f>
@@ -26682,7 +26666,7 @@
     </row>
     <row r="678" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A678" s="21" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B678" s="28" t="s">
         <v>236</v>
@@ -26752,7 +26736,7 @@
     </row>
     <row r="680" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A680" s="21" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B680" s="28" t="s">
         <v>270</v>
@@ -26764,17 +26748,16 @@
         <v>232</v>
       </c>
       <c r="E680" s="22" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F680" s="23" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="G680" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H680" s="25" t="str">
-        <f aca="false">IF(J680&lt;&gt;1,"",IF(I680="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H680" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I680" s="26" t="e">
         <f aca="false">IF(OR(E680="",E680="!!!",F680="NEW"),"",INDEX(B19:B$662,-1+SUMPRODUCT(MAX(ROW(E19:E$662)*(E680=E19:E$662)))))</f>
@@ -26789,7 +26772,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L680" s="29" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
     </row>
     <row r="681" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26831,7 +26814,7 @@
     </row>
     <row r="683" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A683" s="21" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
     </row>
     <row r="684" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26870,7 +26853,7 @@
     </row>
     <row r="685" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A685" s="21" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="E685" s="22" t="str">
         <f aca="false">IF(D685="?OLD","!!!","")</f>
@@ -26904,7 +26887,7 @@
     </row>
     <row r="686" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A686" s="21" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="B686" s="28" t="s">
         <v>243</v>
@@ -27012,7 +26995,7 @@
     </row>
     <row r="689" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A689" s="21" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="B689" s="28" t="s">
         <v>236</v>
@@ -27024,7 +27007,7 @@
         <v>232</v>
       </c>
       <c r="E689" s="22" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="F689" s="23" t="str">
         <f aca="false">IF(OR(E689="",E689="!!!"),"",IF(NOT(ISNA(VLOOKUP(E689,E$1:E688,1,FALSE()))),"OLD",IF(AND(E689&lt;&gt;"",E689&lt;&gt;"!!!"),"NEW","")))</f>
@@ -27050,7 +27033,7 @@
         <v/>
       </c>
       <c r="L689" s="29" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
     </row>
     <row r="690" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27089,7 +27072,7 @@
     </row>
     <row r="691" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A691" s="21" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="E691" s="22" t="str">
         <f aca="false">IF(D691="?OLD","!!!","")</f>
@@ -27123,7 +27106,7 @@
     </row>
     <row r="692" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A692" s="21" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="B692" s="28" t="s">
         <v>270</v>
@@ -27249,9 +27232,8 @@
       <c r="G695" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H695" s="25" t="str">
-        <f aca="false">IF(J695&lt;&gt;1,"",IF(I695="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H695" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I695" s="26" t="str">
         <f aca="false">IF(OR(E695="",E695="!!!",F695="NEW"),"",INDEX(B13:B$683,-1+SUMPRODUCT(MAX(ROW(E13:E$683)*(E695=E13:E$683)))))</f>
@@ -27269,7 +27251,7 @@
     </row>
     <row r="696" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A696" s="21" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="E696" s="22" t="str">
         <f aca="false">IF(D696="?OLD","!!!","")</f>
@@ -27315,7 +27297,7 @@
         <v>232</v>
       </c>
       <c r="E697" s="22" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F697" s="23" t="str">
         <f aca="false">IF(OR(E697="",E697="!!!"),"",IF(NOT(ISNA(VLOOKUP(E697,E$1:E696,1,FALSE()))),"OLD",IF(AND(E697&lt;&gt;"",E697&lt;&gt;"!!!"),"NEW","")))</f>
@@ -27341,12 +27323,12 @@
         <v/>
       </c>
       <c r="L697" s="29" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
     </row>
     <row r="698" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A698" s="21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E698" s="22" t="str">
         <f aca="false">IF(D698="?OLD","!!!","")</f>
@@ -27380,7 +27362,7 @@
     </row>
     <row r="699" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A699" s="21" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="E699" s="22" t="str">
         <f aca="false">IF(D699="?OLD","!!!","")</f>
@@ -27414,7 +27396,7 @@
     </row>
     <row r="700" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A700" s="21" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="B700" s="28" t="s">
         <v>280</v>
@@ -27559,7 +27541,7 @@
     </row>
     <row r="704" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A704" s="21" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="E704" s="22" t="str">
         <f aca="false">IF(D704="?OLD","!!!","")</f>
@@ -27593,10 +27575,10 @@
     </row>
     <row r="705" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A705" s="21" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="B705" s="28" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C705" s="28" t="s">
         <v>351</v>
@@ -27667,7 +27649,7 @@
     </row>
     <row r="707" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A707" s="21" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="E707" s="22" t="str">
         <f aca="false">IF(D707="?OLD","!!!","")</f>
@@ -27701,7 +27683,7 @@
     </row>
     <row r="708" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A708" s="21" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="B708" s="28" t="s">
         <v>342</v>
@@ -27847,7 +27829,7 @@
     </row>
     <row r="712" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A712" s="21" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="E712" s="22" t="str">
         <f aca="false">IF(D712="?OLD","!!!","")</f>
@@ -27881,7 +27863,7 @@
     </row>
     <row r="713" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A713" s="21" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="E713" s="22" t="str">
         <f aca="false">IF(D713="?OLD","!!!","")</f>
@@ -27915,7 +27897,7 @@
     </row>
     <row r="714" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A714" s="21" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="E714" s="22" t="str">
         <f aca="false">IF(D714="?OLD","!!!","")</f>
@@ -27949,7 +27931,7 @@
     </row>
     <row r="715" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A715" s="21" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E715" s="22" t="str">
         <f aca="false">IF(D715="?OLD","!!!","")</f>
@@ -28017,7 +27999,7 @@
     </row>
     <row r="717" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A717" s="21" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E717" s="22" t="str">
         <f aca="false">IF(D717="?OLD","!!!","")</f>
@@ -28060,7 +28042,7 @@
         <v>237</v>
       </c>
       <c r="E718" s="22" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F718" s="23" t="str">
         <f aca="false">IF(OR(E718="",E718="!!!"),"",IF(NOT(ISNA(VLOOKUP(E718,E$1:E717,1,FALSE()))),"OLD",IF(AND(E718&lt;&gt;"",E718&lt;&gt;"!!!"),"NEW","")))</f>
@@ -28086,7 +28068,7 @@
         <v>0</v>
       </c>
       <c r="L718" s="29" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
     </row>
     <row r="719" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28128,12 +28110,12 @@
     </row>
     <row r="721" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A721" s="21" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
     </row>
     <row r="722" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A722" s="21" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E722" s="22" t="str">
         <f aca="false">IF(D722="?OLD","!!!","")</f>
@@ -28167,7 +28149,7 @@
     </row>
     <row r="723" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A723" s="21" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="E723" s="22" t="str">
         <f aca="false">IF(D723="?OLD","!!!","")</f>
@@ -28235,7 +28217,7 @@
     </row>
     <row r="725" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A725" s="21" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="E725" s="22" t="str">
         <f aca="false">IF(D725="?OLD","!!!","")</f>
@@ -28290,9 +28272,8 @@
       <c r="G726" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H726" s="25" t="str">
-        <f aca="false">IF(J726&lt;&gt;1,"",IF(I726="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H726" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I726" s="26" t="n">
         <f aca="false">IF(OR(E726="",E726="!!!",F726="NEW"),"",INDEX(B6:B$721,-1+SUMPRODUCT(MAX(ROW(E6:E$721)*(E726=E6:E$721)))))</f>
@@ -28307,7 +28288,7 @@
         <v>0</v>
       </c>
       <c r="L726" s="29" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
     </row>
     <row r="727" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28346,7 +28327,7 @@
     </row>
     <row r="728" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A728" s="21" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E728" s="22" t="str">
         <f aca="false">IF(D728="?OLD","!!!","")</f>
@@ -28414,7 +28395,7 @@
     </row>
     <row r="730" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A730" s="21" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="E730" s="22" t="str">
         <f aca="false">IF(D730="?OLD","!!!","")</f>
@@ -28520,12 +28501,12 @@
         <v>0</v>
       </c>
       <c r="L732" s="29" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
     </row>
     <row r="733" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A733" s="21" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="E733" s="22" t="str">
         <f aca="false">IF(D733="?OLD","!!!","")</f>
@@ -28559,7 +28540,7 @@
     </row>
     <row r="734" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A734" s="21" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="E734" s="22" t="str">
         <f aca="false">IF(D734="?OLD","!!!","")</f>
@@ -28593,7 +28574,7 @@
     </row>
     <row r="735" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A735" s="21" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="B735" s="28" t="s">
         <v>296</v>
@@ -28664,7 +28645,7 @@
     </row>
     <row r="737" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A737" s="21" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="E737" s="22" t="str">
         <f aca="false">IF(D737="?OLD","!!!","")</f>
@@ -28739,7 +28720,7 @@
     </row>
     <row r="739" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A739" s="21" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="E739" s="22" t="str">
         <f aca="false">IF(D739="?OLD","!!!","")</f>
@@ -28773,7 +28754,7 @@
     </row>
     <row r="740" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A740" s="21" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="B740" s="28" t="s">
         <v>286</v>
@@ -28785,7 +28766,7 @@
         <v>232</v>
       </c>
       <c r="E740" s="22" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F740" s="23" t="str">
         <f aca="false">IF(OR(E740="",E740="!!!"),"",IF(NOT(ISNA(VLOOKUP(E740,E$1:E739,1,FALSE()))),"OLD",IF(AND(E740&lt;&gt;"",E740&lt;&gt;"!!!"),"NEW","")))</f>
@@ -28851,12 +28832,12 @@
     </row>
     <row r="743" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A743" s="21" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
     </row>
     <row r="744" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A744" s="21" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="E744" s="22" t="str">
         <f aca="false">IF(D744="?OLD","!!!","")</f>
@@ -28924,7 +28905,7 @@
     </row>
     <row r="746" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A746" s="21" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="B746" s="28" t="s">
         <v>230</v>
@@ -29016,9 +28997,8 @@
       <c r="G748" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H748" s="25" t="str">
-        <f aca="false">IF(J748&lt;&gt;1,"",IF(I748="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H748" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I748" s="26" t="n">
         <f aca="false">IF(OR(E748="",E748="!!!",F748="NEW"),"",INDEX(B6:B$743,-1+SUMPRODUCT(MAX(ROW(E6:E$743)*(E748=E6:E$743)))))</f>
@@ -29033,12 +29013,12 @@
         <v>0</v>
       </c>
       <c r="L748" s="29" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
     </row>
     <row r="749" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A749" s="21" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B749" s="28" t="s">
         <v>236</v>
@@ -29069,7 +29049,7 @@
     </row>
     <row r="750" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A750" s="21" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="E750" s="22" t="str">
         <f aca="false">IF(D750="?OLD","!!!","")</f>
@@ -29171,7 +29151,7 @@
     </row>
     <row r="753" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A753" s="21" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E753" s="22" t="str">
         <f aca="false">IF(D753="?OLD","!!!","")</f>
@@ -29280,7 +29260,7 @@
     </row>
     <row r="756" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A756" s="21" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="E756" s="22" t="str">
         <f aca="false">IF(D756="?OLD","!!!","")</f>
@@ -29314,7 +29294,7 @@
     </row>
     <row r="757" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A757" s="21" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="E757" s="22" t="str">
         <f aca="false">IF(D757="?OLD","!!!","")</f>
@@ -29382,7 +29362,7 @@
     </row>
     <row r="759" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A759" s="21" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="E759" s="22" t="str">
         <f aca="false">IF(D759="?OLD","!!!","")</f>
@@ -29416,7 +29396,7 @@
     </row>
     <row r="760" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A760" s="21" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="E760" s="22" t="str">
         <f aca="false">IF(D760="?OLD","!!!","")</f>
@@ -29450,7 +29430,7 @@
     </row>
     <row r="761" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A761" s="21" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B761" s="28" t="s">
         <v>236</v>
@@ -29527,12 +29507,12 @@
     </row>
     <row r="764" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A764" s="21" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
     </row>
     <row r="765" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A765" s="21" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="E765" s="22" t="str">
         <f aca="false">IF(D765="?OLD","!!!","")</f>
@@ -29603,7 +29583,7 @@
         <v/>
       </c>
       <c r="L766" s="29" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
     </row>
     <row r="767" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29645,12 +29625,12 @@
     </row>
     <row r="769" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A769" s="21" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
     </row>
     <row r="770" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A770" s="21" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="B770" s="28" t="s">
         <v>230</v>
@@ -29668,9 +29648,8 @@
       <c r="G770" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H770" s="25" t="str">
-        <f aca="false">IF(J770&lt;&gt;1,"",IF(I770="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H770" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I770" s="26" t="str">
         <f aca="false">IF(OR(E770="",E770="!!!",F770="NEW"),"",INDEX(B2:B$769,-1+SUMPRODUCT(MAX(ROW(E2:E$769)*(E770=E2:E$769)))))</f>
@@ -29685,12 +29664,12 @@
         <v>0</v>
       </c>
       <c r="L770" s="29" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
     </row>
     <row r="771" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A771" s="21" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B771" s="28" t="s">
         <v>280</v>
@@ -29761,7 +29740,7 @@
     </row>
     <row r="773" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A773" s="21" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="E773" s="22" t="str">
         <f aca="false">IF(D773="?OLD","!!!","")</f>
@@ -29795,7 +29774,7 @@
     </row>
     <row r="774" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A774" s="21" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="E774" s="22" t="str">
         <f aca="false">IF(D774="?OLD","!!!","")</f>
@@ -29867,7 +29846,7 @@
         <v>0</v>
       </c>
       <c r="L775" s="29" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
     </row>
     <row r="776" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29944,12 +29923,12 @@
         <v>0</v>
       </c>
       <c r="L777" s="29" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
     </row>
     <row r="778" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A778" s="21" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="B778" s="28" t="s">
         <v>236</v>
@@ -29961,7 +29940,7 @@
         <v>232</v>
       </c>
       <c r="E778" s="22" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="F778" s="23" t="s">
         <v>435</v>
@@ -29984,7 +29963,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="L778" s="29" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
     </row>
     <row r="779" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30026,12 +30005,12 @@
     </row>
     <row r="781" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A781" s="21" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
     </row>
     <row r="782" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A782" s="21" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E782" s="22" t="str">
         <f aca="false">IF(D782="?OLD","!!!","")</f>
@@ -30065,7 +30044,7 @@
     </row>
     <row r="783" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A783" s="21" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="E783" s="22" t="str">
         <f aca="false">IF(D783="?OLD","!!!","")</f>
@@ -30099,7 +30078,7 @@
     </row>
     <row r="784" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A784" s="21" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="B784" s="28" t="s">
         <v>270</v>
@@ -30111,10 +30090,10 @@
         <v>232</v>
       </c>
       <c r="E784" s="22" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="F784" s="23" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G784" s="24" t="s">
         <v>287</v>
@@ -30136,12 +30115,12 @@
         <v>#VALUE!</v>
       </c>
       <c r="L784" s="29" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
     </row>
     <row r="785" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A785" s="21" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E785" s="22" t="str">
         <f aca="false">IF(D785="?OLD","!!!","")</f>
@@ -30175,7 +30154,7 @@
     </row>
     <row r="786" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A786" s="21" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="B786" s="28" t="s">
         <v>258</v>
@@ -30187,7 +30166,7 @@
         <v>232</v>
       </c>
       <c r="E786" s="22" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="F786" s="23" t="str">
         <f aca="false">IF(OR(E786="",E786="!!!"),"",IF(NOT(ISNA(VLOOKUP(E786,E$1:E785,1,FALSE()))),"OLD",IF(AND(E786&lt;&gt;"",E786&lt;&gt;"!!!"),"NEW","")))</f>
@@ -30213,12 +30192,12 @@
         <v/>
       </c>
       <c r="L786" s="29" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
     </row>
     <row r="787" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A787" s="21" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="E787" s="22" t="str">
         <f aca="false">IF(D787="?OLD","!!!","")</f>
@@ -30307,9 +30286,8 @@
       <c r="G789" s="24" t="s">
         <v>265</v>
       </c>
-      <c r="H789" s="25" t="str">
-        <f aca="false">IF(J789&lt;&gt;1,"",IF(I789="SBJ","CB","?"))</f>
-        <v/>
+      <c r="H789" s="25" t="s">
+        <v>223</v>
       </c>
       <c r="I789" s="26" t="e">
         <f aca="false">IF(OR(E789="",E789="!!!",F789="NEW"),"",INDEX(B9:B$781,-1+SUMPRODUCT(MAX(ROW(E9:E$781)*(E789=E9:E$781)))))</f>
@@ -30327,7 +30305,7 @@
     </row>
     <row r="790" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A790" s="21" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="E790" s="22" t="str">
         <f aca="false">IF(D790="?OLD","!!!","")</f>
@@ -30429,7 +30407,7 @@
     </row>
     <row r="793" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A793" s="21" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="E793" s="22" t="str">
         <f aca="false">IF(D793="?OLD","!!!","")</f>

</xml_diff>